<commit_message>
PERMANENT GATE STACK in scripts/gate_stack.py - regime(200SMA) + ADX>=20 + DI direction + ZLSMA + liquidity, enforced in code and FAILING CLOSED. evaluate() raises MissingGateData when an input is absent and callers BLOCK rather than pass, because a gate that is documented but not executed is not a gate (SKK was auto-scored PASSING yesterday and caught by hand). og_sweep_runner.js now captures 200/50 SMA, ADX, DI and 20d average dollar volume inline on every sweep so no second forgettable pass is needed. Verified: complete data PASSES, missing ADV RAISES, non-strict BLOCKS, thin ADV BLOCKS. 7/22 rerun through the wired stack reproduces 29 fresh -> 0 with SKK blocked on 84,360 dollar ADV by code.
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-22.xlsx
+++ b/reports/universe_2026-07-22.xlsx
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22 14:55 local</t>
+          <t>2026-07-22 15:02 local</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22 14:55 local</t>
+          <t>2026-07-22 15:02 local</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>$0 - no tradeable name</t>
+          <t>$0 - no name passed the full gate stack</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Full universe read on candles, 155/156 clean. 29 fresh BUY signals culled to 1 by the regime + ADX + DI + ZLSMA stack (SKK), and that one fails liquidity. Net: ZERO tradeable names. Omar stays flat.</t>
+          <t>Full universe read on candles. 29 fresh BUY signals culled to 0 by the regime + ADX + DI + ZLSMA stack.</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
       </c>
       <c r="S4" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-8.05% vs 200-day)</t>
+          <t>BLOCKED: ADX 15.5 below 20</t>
         </is>
       </c>
       <c r="T4" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.05% vs 200-day) - starter size only; ADX 15.5 below 20 - no trend to ride</t>
+          <t>ADX 15.5 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
       </c>
       <c r="S6" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-60.96% vs 200-day)</t>
         </is>
       </c>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - bears in control</t>
+          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="T7" s="11" t="inlineStr">
         <is>
-          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 below ZLSMA 91.2402 - structure has not turned</t>
+          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 at/below ZLSMA 91.2402 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="T8" s="11" t="inlineStr">
         <is>
-          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 below ZLSMA 82.7919 - structure has not turned</t>
+          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 at/below ZLSMA 82.7919 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
       </c>
       <c r="S9" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (70.2% vs 200-day)</t>
+          <t>BLOCKED: -DI 35.0 &gt;= +DI 21.2</t>
         </is>
       </c>
       <c r="T9" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (70.2% vs 200-day) - starter size only; -DI 35.0 &gt;= +DI 21.2 - bears in control</t>
+          <t>-DI 35.0 &gt;= +DI 21.2 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="S10" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (18.77% vs 200-day)</t>
+          <t>BLOCKED: ADX 13.3 below 20</t>
         </is>
       </c>
       <c r="T10" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (18.77% vs 200-day) - starter size only; ADX 13.3 below 20 - no trend to ride</t>
+          <t>ADX 13.3 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="T12" s="11" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - bears in control</t>
+          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="S13" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-29.26% vs 200-day)</t>
         </is>
       </c>
       <c r="T13" s="11" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="T14" s="11" t="inlineStr">
         <is>
-          <t>-DI 27.9 &gt;= +DI 27.0 - bears in control</t>
+          <t>-DI 27.9 &gt;= +DI 27.0 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="S15" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (48.67% vs 200-day)</t>
+          <t>BLOCKED: -DI 32.7 &gt;= +DI 21.5</t>
         </is>
       </c>
       <c r="T15" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (48.67% vs 200-day) - starter size only; -DI 32.7 &gt;= +DI 21.5 - bears in control</t>
+          <t>-DI 32.7 &gt;= +DI 21.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="S16" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-12.4% vs 200-day)</t>
         </is>
       </c>
       <c r="T16" s="11" t="inlineStr">
@@ -2667,12 +2667,12 @@
       </c>
       <c r="S17" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-7.86% vs 200-day)</t>
+          <t>BLOCKED: -DI 31.6 &gt;= +DI 28.1</t>
         </is>
       </c>
       <c r="T17" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-7.86% vs 200-day) - starter size only; -DI 31.6 &gt;= +DI 28.1 - bears in control</t>
+          <t>-DI 31.6 &gt;= +DI 28.1 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="S18" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: liquidity</t>
+          <t>BLOCKED: illiquid</t>
         </is>
       </c>
       <c r="T18" s="11" t="inlineStr">
         <is>
-          <t>Passes regime, ADX 52.4, DI bullish and ZLSMA - the only name to clear the technical stack</t>
+          <t>illiquid - $84,360 avg daily dollar volume; a $85,000 position is 101% of a day's turnover (max $8,436)</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2783,12 @@
       </c>
       <c r="S19" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: price 335.11 below ZLSMA 341.7563</t>
+          <t>BLOCKED: price 335.11 at/below ZLSMA 341.7563</t>
         </is>
       </c>
       <c r="T19" s="11" t="inlineStr">
         <is>
-          <t>price 335.11 below ZLSMA 341.7563 - structure has not turned</t>
+          <t>price 335.11 at/below ZLSMA 341.7563 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2841,12 @@
       </c>
       <c r="S20" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-3.16% vs 200-day)</t>
+          <t>BLOCKED: ADX 12.0 below 20</t>
         </is>
       </c>
       <c r="T20" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-3.16% vs 200-day) - starter size only; ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +D...</t>
+          <t>ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +DI 24.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
       </c>
       <c r="S21" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: price 608.24 below ZLSMA 620.8376</t>
+          <t>BLOCKED: price 608.24 at/below ZLSMA 620.8376</t>
         </is>
       </c>
       <c r="T21" s="11" t="inlineStr">
         <is>
-          <t>price 608.24 below ZLSMA 620.8376 - structure has not turned</t>
+          <t>price 608.24 at/below ZLSMA 620.8376 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
       </c>
       <c r="S22" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-8.97% vs 200-day)</t>
+          <t>BLOCKED: ADX 13.4 below 20</t>
         </is>
       </c>
       <c r="T22" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.97% vs 200-day) - starter size only; ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +D...</t>
+          <t>ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +DI 18.4 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="T23" s="11" t="inlineStr">
         <is>
-          <t>-DI 28.8 &gt;= +DI 20.5 - bears in control; price 28.81 below ZLSMA 30.4577 - structure has not turned</t>
+          <t>-DI 28.8 &gt;= +DI 20.5 - sellers in control; price 28.81 at/below ZLSMA 30.4577 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3073,12 @@
       </c>
       <c r="S24" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: price 75.475 below ZLSMA 78.8225</t>
+          <t>BLOCKED: price 75.475 at/below ZLSMA 78.8225</t>
         </is>
       </c>
       <c r="T24" s="11" t="inlineStr">
         <is>
-          <t>price 75.475 below ZLSMA 78.8225 - structure has not turned</t>
+          <t>price 75.475 at/below ZLSMA 78.8225 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="T26" s="11" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 below ZLSMA 45.596 - structure has not turned</t>
+          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 at/below ZLSMA 45.596 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="T27" s="11" t="inlineStr">
         <is>
-          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 below ZLSMA 374.5233 - structure has not turned</t>
+          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 at/below ZLSMA 374.5233 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3305,12 +3305,12 @@
       </c>
       <c r="S28" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (15.29% vs 200-day)</t>
+          <t>BLOCKED: -DI 25.4 &gt;= +DI 18.4</t>
         </is>
       </c>
       <c r="T28" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (15.29% vs 200-day) - starter size only; -DI 25.4 &gt;= +DI 18.4 - bears in control; price 10.23...</t>
+          <t>-DI 25.4 &gt;= +DI 18.4 - sellers in control; price 10.235 at/below ZLSMA 10.2529 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="S30" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-35.68% vs 200-day)</t>
         </is>
       </c>
       <c r="T30" s="11" t="inlineStr">
@@ -3598,12 +3598,12 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (18.77% vs 200-day)</t>
+          <t>ADX 13.3 below 20</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (18.77% vs 200-day) - starter size only; ADX 13.3 below 20 - no trend to ride</t>
+          <t>ADX 13.3 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -3633,12 +3633,12 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-3.16% vs 200-day)</t>
+          <t>ADX 12.0 below 20</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-3.16% vs 200-day) - starter size only; ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +D...</t>
+          <t>ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +DI 24.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -3668,12 +3668,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>price 608.24 below ZLSMA 620.8376</t>
+          <t>price 608.24 at/below ZLSMA 620.8376</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>price 608.24 below ZLSMA 620.8376 - structure has not turned</t>
+          <t>price 608.24 at/below ZLSMA 620.8376 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3703,12 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.97% vs 200-day)</t>
+          <t>ADX 13.4 below 20</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.97% vs 200-day) - starter size only; ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +D...</t>
+          <t>ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +DI 18.4 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>-DI 28.8 &gt;= +DI 20.5 - bears in control; price 28.81 below ZLSMA 30.4577 - structure has not turned</t>
+          <t>-DI 28.8 &gt;= +DI 20.5 - sellers in control; price 28.81 at/below ZLSMA 30.4577 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3808,12 +3808,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>price 75.475 below ZLSMA 78.8225</t>
+          <t>price 75.475 at/below ZLSMA 78.8225</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>price 75.475 below ZLSMA 78.8225 - structure has not turned</t>
+          <t>price 75.475 at/below ZLSMA 78.8225 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - bears in control</t>
+          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -3878,12 +3878,12 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.05% vs 200-day)</t>
+          <t>ADX 15.5 below 20</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.05% vs 200-day) - starter size only; ADX 15.5 below 20 - no trend to ride</t>
+          <t>ADX 15.5 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 below ZLSMA 45.596 - structure has not turned</t>
+          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 at/below ZLSMA 45.596 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 below ZLSMA 374.5233 - structure has not turned</t>
+          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 at/below ZLSMA 374.5233 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4053,12 +4053,12 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (15.29% vs 200-day)</t>
+          <t>-DI 25.4 &gt;= +DI 18.4</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (15.29% vs 200-day) - starter size only; -DI 25.4 &gt;= +DI 18.4 - bears in control; price 10.23...</t>
+          <t>-DI 25.4 &gt;= +DI 18.4 - sellers in control; price 10.235 at/below ZLSMA 10.2529 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL</t>
+          <t>regime DEEP-FAIL (-29.26% vs 200-day)</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>-DI 27.9 &gt;= +DI 27.0 - bears in control</t>
+          <t>-DI 27.9 &gt;= +DI 27.0 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -4193,12 +4193,12 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (48.67% vs 200-day)</t>
+          <t>-DI 32.7 &gt;= +DI 21.5</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (48.67% vs 200-day) - starter size only; -DI 32.7 &gt;= +DI 21.5 - bears in control</t>
+          <t>-DI 32.7 &gt;= +DI 21.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL</t>
+          <t>regime DEEP-FAIL (-12.4% vs 200-day)</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -4263,12 +4263,12 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-7.86% vs 200-day)</t>
+          <t>-DI 31.6 &gt;= +DI 28.1</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (-7.86% vs 200-day) - starter size only; -DI 31.6 &gt;= +DI 28.1 - bears in control</t>
+          <t>-DI 31.6 &gt;= +DI 28.1 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -4298,12 +4298,12 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL</t>
+          <t>regime DEEP-FAIL (-60.96% vs 200-day)</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - bears in control</t>
+          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL</t>
+          <t>regime DEEP-FAIL (-35.68% vs 200-day)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -4373,7 +4373,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 below ZLSMA 91.2402 - structure has not turned</t>
+          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 at/below ZLSMA 91.2402 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4403,12 +4403,12 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>price 335.11 below ZLSMA 341.7563</t>
+          <t>price 335.11 at/below ZLSMA 341.7563</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>price 335.11 below ZLSMA 341.7563 - structure has not turned</t>
+          <t>price 335.11 at/below ZLSMA 341.7563 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 below ZLSMA 82.7919 - structure has not turned</t>
+          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 at/below ZLSMA 82.7919 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -4473,12 +4473,12 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>liquidity</t>
+          <t>illiquid</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Passes regime, ADX 52.4, DI bullish and ZLSMA - the only name to clear the technical stack</t>
+          <t>illiquid - $84,360 avg daily dollar volume; a $85,000 position is 101% of a day's turnover (max $8,436)</t>
         </is>
       </c>
     </row>
@@ -4508,12 +4508,12 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (70.2% vs 200-day)</t>
+          <t>-DI 35.0 &gt;= +DI 21.2</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>regime REPAIR (70.2% vs 200-day) - starter size only; -DI 35.0 &gt;= +DI 21.2 - bears in control</t>
+          <t>-DI 35.0 &gt;= +DI 21.2 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
       <c r="C2" s="11" t="inlineStr"/>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 below ZLSMA 45.596 - structure has not turned</t>
+          <t>ADX 19.5 below 20 - no trend to ride; price 43.39 at/below ZLSMA 45.596 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       <c r="C4" s="11" t="inlineStr"/>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 below ZLSMA 374.5233 - structure has not turned</t>
+          <t>ADX 18.0 below 20 - no trend to ride; price 367.235 at/below ZLSMA 374.5233 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6347,13 +6347,13 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (15.29% vs 200-day)</t>
+          <t>BLOCKED: -DI 25.4 &gt;= +DI 18.4</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr"/>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (15.29% vs 200-day) - starter size only; -DI 25.4 &gt;= +DI 18.4 - bears in control; price 10.235 below ZLSMA 10.2529 - structure has not turned</t>
+          <t>-DI 25.4 &gt;= +DI 18.4 - sellers in control; price 10.235 at/below ZLSMA 10.2529 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6365,13 +6365,13 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (18.77% vs 200-day)</t>
+          <t>BLOCKED: ADX 13.3 below 20</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr"/>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (18.77% vs 200-day) - starter size only; ADX 13.3 below 20 - no trend to ride</t>
+          <t>ADX 13.3 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -6383,13 +6383,13 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-3.16% vs 200-day)</t>
+          <t>BLOCKED: ADX 12.0 below 20</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr"/>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-3.16% vs 200-day) - starter size only; ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +DI 24.5 - bears in control</t>
+          <t>ADX 12.0 below 20 - no trend to ride; -DI 25.1 &gt;= +DI 24.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6401,13 +6401,13 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-29.26% vs 200-day)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr"/>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL (-29.26% vs 200-day) - watch only, no size; ADX 19.2 below 20 - no trend to ride; -DI 28.3 &gt;= +DI 27.7 - bears in control</t>
+          <t>regime DEEP-FAIL (-29.26% vs 200-day) - watch only, no size; ADX 19.2 below 20 - no trend to ride; -DI 28.3 &gt;= +DI 27.7 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6419,13 +6419,13 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: price 608.24 below ZLSMA 620.8376</t>
+          <t>BLOCKED: price 608.24 at/below ZLSMA 620.8376</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr"/>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>price 608.24 below ZLSMA 620.8376 - structure has not turned</t>
+          <t>price 608.24 at/below ZLSMA 620.8376 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6437,13 +6437,13 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-8.97% vs 200-day)</t>
+          <t>BLOCKED: ADX 13.4 below 20</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr"/>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.97% vs 200-day) - starter size only; ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +DI 18.4 - bears in control</t>
+          <t>ADX 13.4 below 20 - no trend to ride; -DI 19.4 &gt;= +DI 18.4 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
       <c r="C12" s="11" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>-DI 27.9 &gt;= +DI 27.0 - bears in control</t>
+          <t>-DI 27.9 &gt;= +DI 27.0 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       <c r="C13" s="11" t="inlineStr"/>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>-DI 28.8 &gt;= +DI 20.5 - bears in control; price 28.81 below ZLSMA 30.4577 - structure has not turned</t>
+          <t>-DI 28.8 &gt;= +DI 20.5 - sellers in control; price 28.81 at/below ZLSMA 30.4577 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6509,13 +6509,13 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (48.67% vs 200-day)</t>
+          <t>BLOCKED: -DI 32.7 &gt;= +DI 21.5</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (48.67% vs 200-day) - starter size only; -DI 32.7 &gt;= +DI 21.5 - bears in control</t>
+          <t>-DI 32.7 &gt;= +DI 21.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6527,7 +6527,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-12.4% vs 200-day)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr"/>
@@ -6545,13 +6545,13 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-7.86% vs 200-day)</t>
+          <t>BLOCKED: -DI 31.6 &gt;= +DI 28.1</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-7.86% vs 200-day) - starter size only; -DI 31.6 &gt;= +DI 28.1 - bears in control</t>
+          <t>-DI 31.6 &gt;= +DI 28.1 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6581,13 +6581,13 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-60.96% vs 200-day)</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr"/>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - bears in control</t>
+          <t>regime DEEP-FAIL (-60.96% vs 200-day) - watch only, no size; -DI 39.3 &gt;= +DI 17.5 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6599,13 +6599,13 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: price 75.475 below ZLSMA 78.8225</t>
+          <t>BLOCKED: price 75.475 at/below ZLSMA 78.8225</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr"/>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>price 75.475 below ZLSMA 78.8225 - structure has not turned</t>
+          <t>price 75.475 at/below ZLSMA 78.8225 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6617,13 +6617,13 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime DEEP-FAIL</t>
+          <t>BLOCKED: regime DEEP-FAIL (-35.68% vs 200-day)</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>regime DEEP-FAIL (-35.68% vs 200-day) - watch only, no size; ADX 18.9 below 20 - no trend to ride; -DI 26.3 &gt;= +DI 23.3 - bears in control</t>
+          <t>regime DEEP-FAIL (-35.68% vs 200-day) - watch only, no size; ADX 18.9 below 20 - no trend to ride; -DI 26.3 &gt;= +DI 23.3 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       <c r="C21" s="11" t="inlineStr"/>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - bears in control</t>
+          <t>ADX 19.5 below 20 - no trend to ride; -DI 32.1 &gt;= +DI 24.7 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6659,7 +6659,7 @@
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 below ZLSMA 91.2402 - structure has not turned</t>
+          <t>ADX 13.9 below 20 - no trend to ride; price 89.62 at/below ZLSMA 91.2402 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6671,13 +6671,13 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (-8.05% vs 200-day)</t>
+          <t>BLOCKED: ADX 15.5 below 20</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr"/>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (-8.05% vs 200-day) - starter size only; ADX 15.5 below 20 - no trend to ride</t>
+          <t>ADX 15.5 below 20 - no trend to ride</t>
         </is>
       </c>
     </row>
@@ -6689,13 +6689,13 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: price 335.11 below ZLSMA 341.7563</t>
+          <t>BLOCKED: price 335.11 at/below ZLSMA 341.7563</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>price 335.11 below ZLSMA 341.7563 - structure has not turned</t>
+          <t>price 335.11 at/below ZLSMA 341.7563 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6749,7 +6749,7 @@
       <c r="C27" s="11" t="inlineStr"/>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 below ZLSMA 82.7919 - structure has not turned</t>
+          <t>ADX 15.2 below 20 - no trend to ride; price 81.62 at/below ZLSMA 82.7919 - structure has not turned</t>
         </is>
       </c>
     </row>
@@ -6761,13 +6761,13 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: liquidity</t>
+          <t>BLOCKED: illiquid</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Passes regime, ADX 52.4, DI bullish and ZLSMA - the only name to clear the technical stack. DISQUALIFIED ON LIQUIDITY: 20-day average dollar volume is only $84,524. An $85k position would be 100.6% of an entire day's turnover. Today it traded 1,816 shares. Untradeable at this account size regardless of how good the chart looks.</t>
+          <t>illiquid - $84,360 avg daily dollar volume; a $85,000 position is 101% of a day's turnover (max $8,436)</t>
         </is>
       </c>
     </row>
@@ -6797,13 +6797,13 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>BLOCKED: regime REPAIR (70.2% vs 200-day)</t>
+          <t>BLOCKED: -DI 35.0 &gt;= +DI 21.2</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>regime REPAIR (70.2% vs 200-day) - starter size only; -DI 35.0 &gt;= +DI 21.2 - bears in control</t>
+          <t>-DI 35.0 &gt;= +DI 21.2 - sellers in control</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6870,17 +6870,17 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>ZERO tradeable names. 29 fresh signals -&gt; 15 regime PASS -&gt; 6 with ADX&gt;=20 -&gt; 4 DI-bullish -&gt; 1 above ZLSMA (SKK) -&gt; 0 after liquidity.</t>
+          <t>29 fresh Chandelier BUY signals culled to 0. Funnel: fresh signals 29 -&gt; regime PASS 15 -&gt; ADX &gt;= 20 6 -&gt; +DI &gt; -DI 4 -&gt; above ZLSMA 1 -&gt; liquid enough 0.</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>No trades tomorrow. This is the honest output of the scan, not a gap in it.</t>
+          <t>Zero passing names means zero trades - that is the honest output, not a failure of the scan.</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Stay flat. Do not relax a gate to produce a candidate.</t>
+          <t>Do not manufacture a candidate to have something to say.</t>
         </is>
       </c>
     </row>
@@ -6912,73 +6912,23 @@
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>The liquidity gate in build_universe_results.py is defined but NOT wired - MIN_ADV_MULTIPLE is unused because average dollar volume is not in the sweep.</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>SKK was auto-scored as PASSING and had to be disqualified by hand.</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Add average-dollar-volume capture to the sweep reader, then enforce the gate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Gate stack</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>29 fresh Chandelier BUY signals were culled to 1 that pass the full gate stack.</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr"/>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Do not manufacture a candidate to have something to say.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Read on CANDLES on the live chart, per the 2026-07-22 standard.</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr"/>
-      <c r="E6" s="18" t="inlineStr"/>
+      <c r="D4" s="18" t="inlineStr"/>
+      <c r="E4" s="18" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>

</xml_diff>